<commit_message>
ph experimental (config riley)
</commit_message>
<xml_diff>
--- a/res-exp.xlsx
+++ b/res-exp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\Codi\refprop-python-v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ECEFE1B-1BF4-4687-9FBF-DD737A5510BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F01B555-19E4-41FF-88B7-094E13AE5E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{47F7FBFF-A767-4389-BD4D-DADDCD2D5AEE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="113">
   <si>
     <t>Fluido ensayo</t>
   </si>
@@ -372,6 +372,12 @@
   </si>
   <si>
     <t>DME;propylene | 0.85;0.15 Qmass</t>
+  </si>
+  <si>
+    <t>propane_85_DME_15_0_m3_55_65</t>
+  </si>
+  <si>
+    <t>propane;DME | 0.85;0.15 Qmass</t>
   </si>
 </sst>
 </file>
@@ -743,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3411B950-12B0-4E05-A51F-BA853FC747F2}">
-  <dimension ref="A1:CJ9"/>
+  <dimension ref="A1:CJ10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:88" x14ac:dyDescent="0.25">
@@ -754,7 +760,7 @@
         <v>102</v>
       </c>
       <c r="C1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -2679,6 +2685,272 @@
       </c>
       <c r="CJ9">
         <v>8.783729899619043E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:88" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>80.042486645833336</v>
+      </c>
+      <c r="E10">
+        <v>66.037128895833334</v>
+      </c>
+      <c r="F10">
+        <v>25.224740729166665</v>
+      </c>
+      <c r="G10">
+        <v>25.292527848958333</v>
+      </c>
+      <c r="H10">
+        <v>648.87940887560808</v>
+      </c>
+      <c r="I10">
+        <v>369.91974731671246</v>
+      </c>
+      <c r="J10">
+        <v>8.4103770364583337</v>
+      </c>
+      <c r="K10">
+        <v>2.6158610662291863</v>
+      </c>
+      <c r="L10">
+        <v>0.31371547360984309</v>
+      </c>
+      <c r="M10">
+        <v>1.9872976015625028</v>
+      </c>
+      <c r="N10">
+        <v>54.953358395833334</v>
+      </c>
+      <c r="O10">
+        <v>64.978003515624991</v>
+      </c>
+      <c r="P10">
+        <v>230.2605077423292</v>
+      </c>
+      <c r="Q10">
+        <v>272.21034068754904</v>
+      </c>
+      <c r="R10">
+        <v>0.98578055848218127</v>
+      </c>
+      <c r="S10">
+        <v>0.98062806391684176</v>
+      </c>
+      <c r="T10">
+        <v>39.044074906249996</v>
+      </c>
+      <c r="U10">
+        <v>56.197135653869772</v>
+      </c>
+      <c r="V10">
+        <v>338.74254430208333</v>
+      </c>
+      <c r="W10">
+        <v>651.70998102031228</v>
+      </c>
+      <c r="X10">
+        <v>447.32858012386049</v>
+      </c>
+      <c r="Y10">
+        <v>645.53852267840148</v>
+      </c>
+      <c r="Z10">
+        <v>3.703390228870939E-2</v>
+      </c>
+      <c r="AA10">
+        <v>0.31360790358998919</v>
+      </c>
+      <c r="AB10">
+        <v>9.4696391364895438E-3</v>
+      </c>
+      <c r="AC10">
+        <v>1.9239094468131859</v>
+      </c>
+      <c r="AD10">
+        <v>1.3205562385011269</v>
+      </c>
+      <c r="AE10">
+        <v>1.9056907186205818</v>
+      </c>
+      <c r="AF10">
+        <v>1.9234532325424714E-2</v>
+      </c>
+      <c r="AG10">
+        <v>60.065548333333332</v>
+      </c>
+      <c r="AH10">
+        <v>25.292527848958333</v>
+      </c>
+      <c r="AI10">
+        <v>350.09411909235757</v>
+      </c>
+      <c r="AJ10">
+        <v>-0.26851333333333333</v>
+      </c>
+      <c r="AK10">
+        <v>3.7844473020833331</v>
+      </c>
+      <c r="AL10">
+        <v>86.174568760416676</v>
+      </c>
+      <c r="AM10">
+        <v>25.514614697916667</v>
+      </c>
+      <c r="AN10">
+        <v>565.02872451729093</v>
+      </c>
+      <c r="AO10">
+        <v>663.95893689237153</v>
+      </c>
+      <c r="AP10">
+        <v>6.7419659097567317</v>
+      </c>
+      <c r="AQ10">
+        <v>8.4103770364583337</v>
+      </c>
+      <c r="AR10">
+        <v>231.12232954758997</v>
+      </c>
+      <c r="AS10">
+        <v>338.74254430208333</v>
+      </c>
+      <c r="AT10">
+        <v>0.68229495655402539</v>
+      </c>
+      <c r="AU10">
+        <v>2258.6617541524811</v>
+      </c>
+      <c r="AV10">
+        <v>2.1206563264687058E-2</v>
+      </c>
+      <c r="AW10">
+        <v>-6.6672273072916672</v>
+      </c>
+      <c r="AX10">
+        <v>-3.8673248020833335</v>
+      </c>
+      <c r="AY10">
+        <v>3.8821678124999992</v>
+      </c>
+      <c r="AZ10">
+        <v>3.7844473020833331</v>
+      </c>
+      <c r="BA10">
+        <v>350.09411909235757</v>
+      </c>
+      <c r="BB10">
+        <v>559.0250622914599</v>
+      </c>
+      <c r="BC10">
+        <v>2.9174743960249834</v>
+      </c>
+      <c r="BD10">
+        <v>6.5162858647749839</v>
+      </c>
+      <c r="BE10">
+        <v>0.46819722638027894</v>
+      </c>
+      <c r="BF10">
+        <v>8.4103770364583337</v>
+      </c>
+      <c r="BG10">
+        <v>-3.432052083333333E-3</v>
+      </c>
+      <c r="BH10">
+        <v>-2.9424933697916669</v>
+      </c>
+      <c r="BI10">
+        <v>3571.293631891815</v>
+      </c>
+      <c r="BJ10">
+        <v>154.42624691666666</v>
+      </c>
+      <c r="BK10">
+        <v>338.74254430208333</v>
+      </c>
+      <c r="BL10">
+        <v>488.10777969091959</v>
+      </c>
+      <c r="BM10">
+        <v>450.24906767580984</v>
+      </c>
+      <c r="BN10">
+        <v>7.7562197511137201E-2</v>
+      </c>
+      <c r="BO10">
+        <v>1.440940289022673</v>
+      </c>
+      <c r="BP10">
+        <v>1.3291777937237415</v>
+      </c>
+      <c r="BQ10">
+        <v>6</v>
+      </c>
+      <c r="BR10">
+        <v>71</v>
+      </c>
+      <c r="BS10">
+        <v>35.5</v>
+      </c>
+      <c r="BT10">
+        <v>1.4285714285714285E-2</v>
+      </c>
+      <c r="BU10">
+        <v>230</v>
+      </c>
+      <c r="BV10">
+        <v>13.556130016055624</v>
+      </c>
+      <c r="BW10">
+        <v>18.60051557228595</v>
+      </c>
+      <c r="BX10">
+        <v>18.620262027265266</v>
+      </c>
+      <c r="BY10">
+        <v>29.605100887027447</v>
+      </c>
+      <c r="BZ10">
+        <v>4.5861090929466199E-2</v>
+      </c>
+      <c r="CA10">
+        <v>8.7397055330098283E-2</v>
+      </c>
+      <c r="CB10">
+        <v>9.528453593102908E-3</v>
+      </c>
+      <c r="CC10">
+        <v>8.7914940187934928E-2</v>
+      </c>
+      <c r="CD10">
+        <v>4.6132847963688155E-2</v>
+      </c>
+      <c r="CE10">
+        <v>8.1119008323440145</v>
+      </c>
+      <c r="CF10">
+        <v>17.719580150966017</v>
+      </c>
+      <c r="CG10">
+        <v>19.488110627772318</v>
+      </c>
+      <c r="CH10">
+        <v>8.6281669187269934E-3</v>
+      </c>
+      <c r="CI10">
+        <v>6.7310691042362231E-2</v>
+      </c>
+      <c r="CJ10">
+        <v>1.2618159251379723E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>